<commit_message>
chore(session): 세션 마무리 — calibration-plan confirm-all + NC 워크플로우 + manage-skills 업데이트
- calibration-plans: confirm-all API 엔드포인트 추가, CalibrationDate payload 필드 보강
- calibration-plan: UL-QP-19-01(00) xlsx 양식 교체 반영, layout 주석 갱신
- calibration-plan-sync.listener: 교정 완료 이벤트→계획 항목 연동 리스너 추가
- harness 산출물: nc-workflow-atomicity/event-payload-ssot-fix/calibration-plan-confirm 계약·평가 추가
- manage-skills: verify-handover-security + verify-qr-ssot 등록 누락 복구 (2개 스킬)
- verify-sql-safety: Step 10 추가 — as const 배열 Drizzle spread 누락 탐지
- verify-cache-events: Step 5a 추가 — 이벤트 페이로드 완전성 검사
- verify-implementation: 17·18번 스킬 추가 (handover-security + qr-ssot)
- harness-docs: 아카이브 references 추가 (domain/export/index/infra/migration)
- tech-debt-tracker: 이번 세션 발견 기술 부채 항목 기록

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/procedure/template/UL-QP-19-01(00) 연간 교정계획서.xlsx
+++ b/docs/procedure/template/UL-QP-19-01(00) 연간 교정계획서.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmjkd\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E290C9BF-F954-4F44-8E25-CF49760EDF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFB873E-0C8D-46B9-B175-4142E4123E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2412" yWindow="2508" windowWidth="23040" windowHeight="13560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1010,48 +1010,6 @@
     <xf numFmtId="176" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1089,6 +1047,48 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1489,73 +1489,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" thickBot="1">
-      <c r="A3" s="35"/>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
     </row>
     <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38" t="s">
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38"/>
-      <c r="J4" s="31" t="s">
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="17" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1" thickBot="1">
-      <c r="A5" s="37"/>
+      <c r="A5" s="23"/>
       <c r="B5" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="39"/>
+      <c r="C5" s="25"/>
       <c r="D5" s="10" t="s">
         <v>12</v>
       </c>
@@ -1574,7 +1574,7 @@
       <c r="I5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="32"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="7">
@@ -1959,61 +1959,61 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="2"/>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D34" s="28"/>
-      <c r="E34" s="27" t="s">
+      <c r="D34" s="14"/>
+      <c r="E34" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F34" s="28"/>
-      <c r="G34" s="27" t="s">
+      <c r="F34" s="14"/>
+      <c r="G34" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="H34" s="28"/>
-      <c r="I34" s="27" t="s">
+      <c r="H34" s="14"/>
+      <c r="I34" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="J34" s="29"/>
+      <c r="J34" s="15"/>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="2"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="14"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="26"/>
+      <c r="J35" s="27"/>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="2"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="15"/>
-      <c r="J36" s="16"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="29"/>
     </row>
     <row r="37" spans="1:10" ht="14.4" thickBot="1">
       <c r="A37" s="2"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="17" t="s">
+      <c r="C37" s="36"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F37" s="26"/>
-      <c r="G37" s="17" t="s">
+      <c r="F37" s="39"/>
+      <c r="G37" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="H37" s="26"/>
-      <c r="I37" s="17" t="s">
+      <c r="H37" s="39"/>
+      <c r="I37" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="J37" s="18"/>
+      <c r="J37" s="31"/>
     </row>
     <row r="38" spans="1:10" ht="17.399999999999999">
       <c r="A38" s="8" t="s">
@@ -2047,7 +2047,14 @@
     <filterColumn colId="7" showButton="0"/>
     <filterColumn colId="8" showButton="0"/>
   </autoFilter>
-  <mergeCells count="20">
+  <mergeCells count="17">
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="C35:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="E35:F36"/>
+    <mergeCell ref="G35:H36"/>
+    <mergeCell ref="I35:J36"/>
     <mergeCell ref="G34:H34"/>
     <mergeCell ref="I34:J34"/>
     <mergeCell ref="C34:D34"/>
@@ -2058,16 +2065,6 @@
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="E34:F34"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="C35:D37"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="G37:H37"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -2083,12 +2080,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2315,15 +2309,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D850C4EC-85E4-47B7-A821-A2BA677C1E30}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99E5F957-E121-4724-8A88-C84B114DD49F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f64d2594-2a84-4999-a7b8-49648faa3cbd"/>
+    <ds:schemaRef ds:uri="fff104b8-6195-4b91-b705-97690b5c6b25"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2348,18 +2354,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99E5F957-E121-4724-8A88-C84B114DD49F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D850C4EC-85E4-47B7-A821-A2BA677C1E30}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f64d2594-2a84-4999-a7b8-49648faa3cbd"/>
-    <ds:schemaRef ds:uri="fff104b8-6195-4b91-b705-97690b5c6b25"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>